<commit_message>
Added new RDF data schemes and visual schemes for economy-table75-79, and fixed XLSX spreadsheets for economy-table75-76
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table75.xlsx
+++ b/sources/table_normalization/xlsx/economy-table75.xlsx
@@ -337,11 +337,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="167" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
-    <numFmt numFmtId="171" formatCode="[$-409]mmmm\-yy;@"/>
+    <numFmt numFmtId="164" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
+    <numFmt numFmtId="168" formatCode="[$-409]mmmm\-yy;@"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -566,12 +566,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -581,7 +581,7 @@
     <xf numFmtId="17" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -590,7 +590,7 @@
     <xf numFmtId="17" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -602,34 +602,31 @@
     <xf numFmtId="17" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="5" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="4" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="4" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -644,7 +641,7 @@
     <xf numFmtId="17" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -665,19 +662,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="17" fontId="6" fillId="10" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="6" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -692,43 +686,124 @@
     <xf numFmtId="17" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="10" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="2" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="17" fontId="10" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -737,100 +812,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -845,16 +845,28 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="10" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="6" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -865,7 +877,7 @@
   </cellStyles>
   <dxfs count="27">
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
@@ -873,7 +885,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FF92D050"/>
@@ -881,7 +893,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
@@ -889,7 +901,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FF92D050"/>
@@ -897,7 +909,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
@@ -905,7 +917,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FF92D050"/>
@@ -913,7 +925,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
@@ -921,7 +933,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FF92D050"/>
@@ -929,7 +941,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FF92D050"/>
@@ -937,7 +949,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[$-409]mmm\-yy;@"/>
+      <numFmt numFmtId="167" formatCode="[$-409]mmm\-yy;@"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
@@ -1448,85 +1460,85 @@
       </c>
       <c r="J1" s="89"/>
       <c r="K1" s="89"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
     </row>
     <row r="2" spans="1:16" ht="15.5">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="91" t="s">
+      <c r="B2" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="91" t="s">
+      <c r="C2" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="91" t="s">
+      <c r="D2" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="91" t="s">
+      <c r="E2" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="91" t="s">
+      <c r="F2" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="91" t="s">
+      <c r="G2" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="91" t="s">
+      <c r="H2" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="91" t="s">
+      <c r="I2" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="91" t="s">
+      <c r="J2" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="92" t="s">
+      <c r="K2" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="93">
+      <c r="L2" s="98">
         <v>1</v>
       </c>
-      <c r="M2" s="93">
+      <c r="M2" s="98">
         <v>2</v>
       </c>
-      <c r="N2" s="93">
+      <c r="N2" s="98">
         <v>3</v>
       </c>
-      <c r="O2" s="93" t="s">
+      <c r="O2" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="93" t="s">
+      <c r="P2" s="44" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15.5">
-      <c r="A3" s="45">
+      <c r="A3" s="77">
         <v>1</v>
       </c>
-      <c r="B3" s="45">
+      <c r="B3" s="77">
         <v>1</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="45" t="s">
+      <c r="F3" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="45" t="s">
+      <c r="G3" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="45">
+      <c r="H3" s="77">
         <v>121</v>
       </c>
       <c r="I3" s="1">
@@ -1538,65 +1550,65 @@
       <c r="K3" s="3">
         <v>41426</v>
       </c>
-      <c r="L3" s="55">
+      <c r="L3" s="53">
         <v>187200</v>
       </c>
-      <c r="M3" s="55">
+      <c r="M3" s="53">
         <v>0</v>
       </c>
-      <c r="N3" s="55">
+      <c r="N3" s="53">
         <v>748800</v>
       </c>
-      <c r="O3" s="55">
+      <c r="O3" s="53">
         <v>0.25</v>
       </c>
-      <c r="P3" s="55">
+      <c r="P3" s="53">
         <v>936000</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.5">
-      <c r="A4" s="45"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
+      <c r="A4" s="77"/>
+      <c r="B4" s="77"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
       <c r="I4" s="4">
         <v>41244</v>
       </c>
       <c r="J4" s="5"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="56"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="56"/>
-      <c r="P4" s="56"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="54"/>
+      <c r="N4" s="54"/>
+      <c r="O4" s="54"/>
+      <c r="P4" s="54"/>
     </row>
     <row r="5" spans="1:16" ht="15.5">
-      <c r="A5" s="45">
+      <c r="A5" s="77">
         <v>2</v>
       </c>
-      <c r="B5" s="45">
+      <c r="B5" s="77">
         <v>1</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="45" t="s">
+      <c r="E5" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="F5" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="45">
+      <c r="H5" s="77">
         <v>127</v>
       </c>
       <c r="I5" s="1">
@@ -1608,69 +1620,69 @@
       <c r="K5" s="3">
         <v>41334</v>
       </c>
-      <c r="L5" s="55">
+      <c r="L5" s="53">
         <v>62000</v>
       </c>
-      <c r="M5" s="55">
+      <c r="M5" s="53">
         <v>346320</v>
       </c>
-      <c r="N5" s="55" t="s">
+      <c r="N5" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="O5" s="55">
+      <c r="O5" s="53">
         <v>1</v>
       </c>
-      <c r="P5" s="55">
+      <c r="P5" s="53">
         <v>408320</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="15.5">
-      <c r="A6" s="45"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
+      <c r="A6" s="77"/>
+      <c r="B6" s="77"/>
+      <c r="C6" s="84"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
       <c r="I6" s="7">
         <v>41183</v>
       </c>
       <c r="J6" s="8">
         <v>41426</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="97">
         <v>41609</v>
       </c>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="56"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
+      <c r="L6" s="54"/>
+      <c r="M6" s="54"/>
+      <c r="N6" s="54"/>
+      <c r="O6" s="54"/>
+      <c r="P6" s="54"/>
     </row>
     <row r="7" spans="1:16" ht="15.5">
-      <c r="A7" s="45">
+      <c r="A7" s="77">
         <v>2</v>
       </c>
-      <c r="B7" s="45">
+      <c r="B7" s="77">
         <v>1</v>
       </c>
-      <c r="C7" s="46" t="s">
+      <c r="C7" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="45" t="s">
+      <c r="E7" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="45" t="s">
+      <c r="F7" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="45">
+      <c r="H7" s="77">
         <v>512</v>
       </c>
       <c r="I7" s="1">
@@ -1682,65 +1694,65 @@
       <c r="K7" s="3">
         <v>41395</v>
       </c>
-      <c r="L7" s="55">
+      <c r="L7" s="53">
         <v>93000</v>
       </c>
-      <c r="M7" s="55">
+      <c r="M7" s="53">
         <v>499500</v>
       </c>
-      <c r="N7" s="55" t="s">
+      <c r="N7" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="O7" s="55">
+      <c r="O7" s="53">
         <v>0.5</v>
       </c>
-      <c r="P7" s="55">
+      <c r="P7" s="53">
         <v>592500</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15.5">
-      <c r="A8" s="45"/>
-      <c r="B8" s="45"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
+      <c r="A8" s="77"/>
+      <c r="B8" s="77"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="77"/>
+      <c r="E8" s="77"/>
+      <c r="F8" s="77"/>
+      <c r="G8" s="77"/>
+      <c r="H8" s="77"/>
       <c r="I8" s="7">
         <v>41214</v>
       </c>
       <c r="J8" s="9"/>
       <c r="K8" s="10"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="56"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="56"/>
-      <c r="P8" s="56"/>
+      <c r="L8" s="54"/>
+      <c r="M8" s="54"/>
+      <c r="N8" s="54"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="54"/>
     </row>
     <row r="9" spans="1:16" ht="15.5">
-      <c r="A9" s="45">
+      <c r="A9" s="77">
         <v>2</v>
       </c>
-      <c r="B9" s="45">
+      <c r="B9" s="77">
         <v>1</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="C9" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="45" t="s">
+      <c r="E9" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="45" t="s">
+      <c r="F9" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="45">
+      <c r="H9" s="77">
         <v>619</v>
       </c>
       <c r="I9" s="1">
@@ -1752,65 +1764,65 @@
       <c r="K9" s="3">
         <v>41487</v>
       </c>
-      <c r="L9" s="55">
+      <c r="L9" s="53">
         <v>57600</v>
       </c>
-      <c r="M9" s="55" t="s">
+      <c r="M9" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="N9" s="55" t="s">
+      <c r="N9" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="55">
+      <c r="O9" s="53">
         <v>0.5</v>
       </c>
-      <c r="P9" s="55">
+      <c r="P9" s="53">
         <v>57600</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.5">
-      <c r="A10" s="45"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
+      <c r="A10" s="77"/>
+      <c r="B10" s="77"/>
+      <c r="C10" s="84"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
       <c r="I10" s="7">
         <v>41214</v>
       </c>
       <c r="J10" s="9"/>
       <c r="K10" s="10"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="56"/>
-      <c r="N10" s="56"/>
-      <c r="O10" s="56"/>
-      <c r="P10" s="56"/>
+      <c r="L10" s="54"/>
+      <c r="M10" s="54"/>
+      <c r="N10" s="54"/>
+      <c r="O10" s="54"/>
+      <c r="P10" s="54"/>
     </row>
     <row r="11" spans="1:16" ht="15.5">
-      <c r="A11" s="45">
+      <c r="A11" s="77">
         <v>2</v>
       </c>
-      <c r="B11" s="45">
+      <c r="B11" s="77">
         <v>2</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="45" t="s">
+      <c r="E11" s="77" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="45" t="s">
+      <c r="F11" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="45" t="s">
+      <c r="G11" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="45">
+      <c r="H11" s="77">
         <v>847</v>
       </c>
       <c r="I11" s="1">
@@ -1822,65 +1834,65 @@
       <c r="K11" s="3">
         <v>41456</v>
       </c>
-      <c r="L11" s="55" t="s">
+      <c r="L11" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="M11" s="55" t="s">
+      <c r="M11" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="N11" s="55" t="s">
+      <c r="N11" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="O11" s="55">
+      <c r="O11" s="53">
         <v>0.5</v>
       </c>
-      <c r="P11" s="55" t="s">
+      <c r="P11" s="53" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="15.5">
-      <c r="A12" s="45"/>
-      <c r="B12" s="45"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
+      <c r="A12" s="77"/>
+      <c r="B12" s="77"/>
+      <c r="C12" s="84"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
       <c r="I12" s="7">
         <v>41275</v>
       </c>
       <c r="J12" s="9"/>
       <c r="K12" s="10"/>
-      <c r="L12" s="56"/>
-      <c r="M12" s="56"/>
-      <c r="N12" s="56"/>
-      <c r="O12" s="56"/>
-      <c r="P12" s="56"/>
+      <c r="L12" s="54"/>
+      <c r="M12" s="54"/>
+      <c r="N12" s="54"/>
+      <c r="O12" s="54"/>
+      <c r="P12" s="54"/>
     </row>
     <row r="13" spans="1:16" ht="15.5">
-      <c r="A13" s="45">
+      <c r="A13" s="77">
         <v>2</v>
       </c>
-      <c r="B13" s="45">
+      <c r="B13" s="77">
         <v>1</v>
       </c>
-      <c r="C13" s="46" t="s">
+      <c r="C13" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="45" t="s">
+      <c r="D13" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="45" t="s">
+      <c r="E13" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="45" t="s">
+      <c r="F13" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="45" t="s">
+      <c r="G13" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="45">
+      <c r="H13" s="77">
         <v>156</v>
       </c>
       <c r="I13" s="1">
@@ -1892,65 +1904,65 @@
       <c r="K13" s="12">
         <v>41030</v>
       </c>
-      <c r="L13" s="55" t="s">
+      <c r="L13" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="M13" s="55" t="s">
+      <c r="M13" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="N13" s="55" t="s">
+      <c r="N13" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="O13" s="55">
+      <c r="O13" s="53">
         <v>0.33</v>
       </c>
-      <c r="P13" s="55" t="s">
+      <c r="P13" s="53" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="15.5">
-      <c r="A14" s="45"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
+      <c r="A14" s="77"/>
+      <c r="B14" s="77"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
       <c r="I14" s="13">
         <v>41214</v>
       </c>
       <c r="J14" s="9"/>
       <c r="K14" s="9"/>
-      <c r="L14" s="56"/>
-      <c r="M14" s="56"/>
-      <c r="N14" s="56"/>
-      <c r="O14" s="56"/>
-      <c r="P14" s="56"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="54"/>
+      <c r="N14" s="54"/>
+      <c r="O14" s="54"/>
+      <c r="P14" s="54"/>
     </row>
     <row r="15" spans="1:16" ht="15.5">
-      <c r="A15" s="45">
+      <c r="A15" s="77">
         <v>1</v>
       </c>
-      <c r="B15" s="45">
+      <c r="B15" s="77">
         <v>1</v>
       </c>
-      <c r="C15" s="46" t="s">
+      <c r="C15" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="45" t="s">
+      <c r="E15" s="77" t="s">
         <v>33</v>
       </c>
-      <c r="F15" s="45" t="s">
+      <c r="F15" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="45" t="s">
+      <c r="G15" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="45">
+      <c r="H15" s="77">
         <v>848</v>
       </c>
       <c r="I15" s="1">
@@ -1962,69 +1974,69 @@
       <c r="K15" s="14">
         <v>41334</v>
       </c>
-      <c r="L15" s="55">
+      <c r="L15" s="53">
         <v>379260</v>
       </c>
-      <c r="M15" s="55">
+      <c r="M15" s="53">
         <v>1905000</v>
       </c>
-      <c r="N15" s="55">
+      <c r="N15" s="53">
         <v>0</v>
       </c>
-      <c r="O15" s="55">
+      <c r="O15" s="53">
         <v>1</v>
       </c>
-      <c r="P15" s="55">
+      <c r="P15" s="53">
         <v>2284260</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="15.5">
-      <c r="A16" s="45"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="45"/>
+      <c r="A16" s="77"/>
+      <c r="B16" s="77"/>
+      <c r="C16" s="84"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
       <c r="I16" s="4">
         <v>41091</v>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="96">
         <v>41306</v>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="15">
         <v>41426</v>
       </c>
-      <c r="L16" s="56"/>
-      <c r="M16" s="56"/>
-      <c r="N16" s="56"/>
-      <c r="O16" s="56"/>
-      <c r="P16" s="56"/>
+      <c r="L16" s="54"/>
+      <c r="M16" s="54"/>
+      <c r="N16" s="54"/>
+      <c r="O16" s="54"/>
+      <c r="P16" s="54"/>
     </row>
     <row r="17" spans="1:16" ht="15.5">
-      <c r="A17" s="45">
+      <c r="A17" s="77">
         <v>1</v>
       </c>
-      <c r="B17" s="45">
+      <c r="B17" s="77">
         <v>1</v>
       </c>
-      <c r="C17" s="46" t="s">
+      <c r="C17" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="D17" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="E17" s="45" t="s">
+      <c r="E17" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="F17" s="45" t="s">
+      <c r="F17" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G17" s="45" t="s">
+      <c r="G17" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="45">
+      <c r="H17" s="77">
         <v>265</v>
       </c>
       <c r="I17" s="1">
@@ -2033,66 +2045,66 @@
       <c r="J17" s="2">
         <v>41456</v>
       </c>
-      <c r="K17" s="14">
+      <c r="K17" s="95">
         <v>41487</v>
       </c>
-      <c r="L17" s="55">
+      <c r="L17" s="53">
         <v>91760</v>
       </c>
-      <c r="M17" s="55">
+      <c r="M17" s="53">
         <v>479520</v>
       </c>
-      <c r="N17" s="55">
+      <c r="N17" s="53">
         <v>0</v>
       </c>
-      <c r="O17" s="55">
+      <c r="O17" s="53">
         <v>0.75</v>
       </c>
-      <c r="P17" s="55">
+      <c r="P17" s="53">
         <v>571280</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="15.5">
-      <c r="A18" s="45"/>
-      <c r="B18" s="45"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="17"/>
+      <c r="A18" s="77"/>
+      <c r="B18" s="77"/>
+      <c r="C18" s="84"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="77"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="16"/>
       <c r="J18" s="11"/>
       <c r="K18" s="12"/>
-      <c r="L18" s="56"/>
-      <c r="M18" s="56"/>
-      <c r="N18" s="56"/>
-      <c r="O18" s="56"/>
-      <c r="P18" s="56"/>
+      <c r="L18" s="54"/>
+      <c r="M18" s="54"/>
+      <c r="N18" s="54"/>
+      <c r="O18" s="54"/>
+      <c r="P18" s="54"/>
     </row>
     <row r="19" spans="1:16" ht="15.5">
-      <c r="A19" s="46">
+      <c r="A19" s="83">
         <v>1</v>
       </c>
-      <c r="B19" s="46">
+      <c r="B19" s="83">
         <v>1</v>
       </c>
-      <c r="C19" s="46" t="s">
+      <c r="C19" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="46" t="s">
+      <c r="D19" s="83" t="s">
         <v>37</v>
       </c>
-      <c r="E19" s="46" t="s">
+      <c r="E19" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="46" t="s">
+      <c r="F19" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G19" s="46" t="s">
+      <c r="G19" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="H19" s="46" t="s">
+      <c r="H19" s="83" t="s">
         <v>40</v>
       </c>
       <c r="I19" s="2">
@@ -2101,292 +2113,292 @@
       <c r="J19" s="2">
         <v>41334</v>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="17">
         <v>41426</v>
       </c>
-      <c r="L19" s="57">
+      <c r="L19" s="74">
         <v>148800</v>
       </c>
-      <c r="M19" s="57">
+      <c r="M19" s="74">
         <v>397800</v>
       </c>
-      <c r="N19" s="57">
+      <c r="N19" s="74">
         <v>0</v>
       </c>
-      <c r="O19" s="68">
+      <c r="O19" s="65">
         <v>1</v>
       </c>
-      <c r="P19" s="81">
+      <c r="P19" s="48">
         <v>546600</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="15.5">
-      <c r="A20" s="47"/>
-      <c r="B20" s="47"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
+      <c r="A20" s="84"/>
+      <c r="B20" s="84"/>
+      <c r="C20" s="84"/>
+      <c r="D20" s="84"/>
+      <c r="E20" s="84"/>
+      <c r="F20" s="84"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="84"/>
       <c r="I20" s="8">
         <v>40817</v>
       </c>
-      <c r="J20" s="19">
+      <c r="J20" s="18">
         <v>41091</v>
       </c>
-      <c r="K20" s="6">
+      <c r="K20" s="93">
         <v>41456</v>
       </c>
-      <c r="L20" s="57"/>
-      <c r="M20" s="57"/>
-      <c r="N20" s="57"/>
-      <c r="O20" s="68"/>
-      <c r="P20" s="81"/>
+      <c r="L20" s="74"/>
+      <c r="M20" s="74"/>
+      <c r="N20" s="74"/>
+      <c r="O20" s="65"/>
+      <c r="P20" s="48"/>
     </row>
     <row r="21" spans="1:16" ht="15.5">
-      <c r="A21" s="46">
+      <c r="A21" s="83">
         <v>2</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="83">
         <v>1</v>
       </c>
-      <c r="C21" s="46" t="s">
+      <c r="C21" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="46" t="s">
+      <c r="D21" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="E21" s="46" t="s">
+      <c r="E21" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="46" t="s">
+      <c r="F21" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G21" s="46" t="s">
+      <c r="G21" s="83" t="s">
         <v>43</v>
       </c>
-      <c r="H21" s="46" t="s">
+      <c r="H21" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="I21" s="20">
+      <c r="I21" s="19">
         <v>41275</v>
       </c>
-      <c r="J21" s="20">
+      <c r="J21" s="19">
         <v>41365</v>
       </c>
-      <c r="K21" s="20">
+      <c r="K21" s="19">
         <v>41334</v>
       </c>
-      <c r="L21" s="57">
+      <c r="L21" s="74">
         <v>0</v>
       </c>
-      <c r="M21" s="57">
+      <c r="M21" s="74">
         <v>0</v>
       </c>
-      <c r="N21" s="57">
+      <c r="N21" s="74">
         <v>540000</v>
       </c>
-      <c r="O21" s="68">
+      <c r="O21" s="65">
         <v>1</v>
       </c>
-      <c r="P21" s="81">
+      <c r="P21" s="48">
         <v>540000</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="15.5">
-      <c r="A22" s="47"/>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="21">
+      <c r="A22" s="84"/>
+      <c r="B22" s="84"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="84"/>
+      <c r="E22" s="84"/>
+      <c r="F22" s="84"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="84"/>
+      <c r="I22" s="20">
         <v>41275</v>
       </c>
-      <c r="J22" s="21">
+      <c r="J22" s="20">
         <v>41306</v>
       </c>
-      <c r="K22" s="21">
+      <c r="K22" s="20">
         <v>41306</v>
       </c>
-      <c r="L22" s="57"/>
-      <c r="M22" s="57"/>
-      <c r="N22" s="57"/>
-      <c r="O22" s="68"/>
-      <c r="P22" s="81"/>
+      <c r="L22" s="74"/>
+      <c r="M22" s="74"/>
+      <c r="N22" s="74"/>
+      <c r="O22" s="65"/>
+      <c r="P22" s="48"/>
     </row>
     <row r="23" spans="1:16" ht="15.5">
-      <c r="A23" s="46">
+      <c r="A23" s="83">
         <v>2</v>
       </c>
-      <c r="B23" s="46">
+      <c r="B23" s="83">
         <v>1</v>
       </c>
-      <c r="C23" s="46" t="s">
+      <c r="C23" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D23" s="46" t="s">
+      <c r="D23" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="46" t="s">
+      <c r="E23" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="46" t="s">
+      <c r="F23" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G23" s="46" t="s">
+      <c r="G23" s="83" t="s">
         <v>43</v>
       </c>
-      <c r="H23" s="46" t="s">
+      <c r="H23" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="I23" s="20">
+      <c r="I23" s="19">
         <v>41306</v>
       </c>
-      <c r="J23" s="20">
+      <c r="J23" s="19">
         <v>41852</v>
       </c>
-      <c r="K23" s="20">
+      <c r="K23" s="19">
         <v>41699</v>
       </c>
-      <c r="L23" s="55">
+      <c r="L23" s="53">
         <v>44640</v>
       </c>
-      <c r="M23" s="55">
+      <c r="M23" s="53">
         <v>119340</v>
       </c>
-      <c r="N23" s="55">
+      <c r="N23" s="53">
         <v>0</v>
       </c>
-      <c r="O23" s="69">
+      <c r="O23" s="66">
         <v>0.5</v>
       </c>
-      <c r="P23" s="81">
+      <c r="P23" s="48">
         <v>163980</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="15.5">
-      <c r="A24" s="47"/>
-      <c r="B24" s="47"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="47"/>
-      <c r="I24" s="22">
+      <c r="A24" s="84"/>
+      <c r="B24" s="84"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="84"/>
+      <c r="E24" s="84"/>
+      <c r="F24" s="84"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="84"/>
+      <c r="I24" s="21">
         <v>41334</v>
       </c>
-      <c r="J24" s="23">
+      <c r="J24" s="22">
         <v>41852</v>
       </c>
-      <c r="K24" s="23">
+      <c r="K24" s="22">
         <v>41699</v>
       </c>
-      <c r="L24" s="56"/>
-      <c r="M24" s="56"/>
-      <c r="N24" s="56"/>
-      <c r="O24" s="70"/>
-      <c r="P24" s="81"/>
+      <c r="L24" s="54"/>
+      <c r="M24" s="54"/>
+      <c r="N24" s="54"/>
+      <c r="O24" s="67"/>
+      <c r="P24" s="48"/>
     </row>
     <row r="25" spans="1:16" ht="15.5">
-      <c r="A25" s="46">
+      <c r="A25" s="83">
         <v>2</v>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="83">
         <v>1</v>
       </c>
-      <c r="C25" s="46" t="s">
+      <c r="C25" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="E25" s="46" t="s">
+      <c r="E25" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="F25" s="46" t="s">
+      <c r="F25" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G25" s="46" t="s">
+      <c r="G25" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="H25" s="46" t="s">
+      <c r="H25" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="I25" s="20">
+      <c r="I25" s="19">
         <v>41395</v>
       </c>
-      <c r="J25" s="20">
+      <c r="J25" s="19">
         <v>41671</v>
       </c>
-      <c r="K25" s="20">
+      <c r="K25" s="19">
         <v>41640</v>
       </c>
-      <c r="L25" s="55">
+      <c r="L25" s="53">
         <v>411744</v>
       </c>
-      <c r="M25" s="55">
+      <c r="M25" s="53">
         <v>0</v>
       </c>
-      <c r="N25" s="55">
+      <c r="N25" s="53">
         <v>1205900</v>
       </c>
-      <c r="O25" s="69">
+      <c r="O25" s="66">
         <v>0.5</v>
       </c>
-      <c r="P25" s="81">
+      <c r="P25" s="48">
         <v>1617644</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="15.5">
-      <c r="A26" s="47"/>
-      <c r="B26" s="47"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="20">
+      <c r="A26" s="84"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="84"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="84"/>
+      <c r="G26" s="84"/>
+      <c r="H26" s="84"/>
+      <c r="I26" s="19">
         <v>41456</v>
       </c>
-      <c r="J26" s="23">
+      <c r="J26" s="22">
         <v>41671</v>
       </c>
-      <c r="K26" s="23">
+      <c r="K26" s="22">
         <v>41640</v>
       </c>
-      <c r="L26" s="56"/>
-      <c r="M26" s="56"/>
-      <c r="N26" s="56"/>
-      <c r="O26" s="70"/>
-      <c r="P26" s="81"/>
+      <c r="L26" s="54"/>
+      <c r="M26" s="54"/>
+      <c r="N26" s="54"/>
+      <c r="O26" s="67"/>
+      <c r="P26" s="48"/>
     </row>
     <row r="27" spans="1:16" ht="15.5">
-      <c r="A27" s="46"/>
-      <c r="B27" s="46">
+      <c r="A27" s="83"/>
+      <c r="B27" s="83">
         <v>1</v>
       </c>
-      <c r="C27" s="46" t="s">
+      <c r="C27" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="E27" s="46" t="s">
+      <c r="E27" s="83" t="s">
         <v>48</v>
       </c>
-      <c r="F27" s="46" t="s">
+      <c r="F27" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G27" s="46" t="s">
+      <c r="G27" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="H27" s="46" t="s">
+      <c r="H27" s="83" t="s">
         <v>40</v>
       </c>
       <c r="I27" s="2">
@@ -2395,178 +2407,178 @@
       <c r="J27" s="2">
         <v>41306</v>
       </c>
-      <c r="K27" s="18">
+      <c r="K27" s="17">
         <v>41426</v>
       </c>
-      <c r="L27" s="57">
+      <c r="L27" s="74">
         <v>0</v>
       </c>
-      <c r="M27" s="57">
+      <c r="M27" s="74">
         <v>0</v>
       </c>
-      <c r="N27" s="57">
+      <c r="N27" s="74">
         <v>18000</v>
       </c>
-      <c r="O27" s="68">
+      <c r="O27" s="65">
         <v>0.3</v>
       </c>
-      <c r="P27" s="81">
+      <c r="P27" s="48">
         <v>18000</v>
       </c>
     </row>
     <row r="28" spans="1:16" ht="15.5">
-      <c r="A28" s="47"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="47"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
-      <c r="I28" s="22">
+      <c r="A28" s="84"/>
+      <c r="B28" s="84"/>
+      <c r="C28" s="84"/>
+      <c r="D28" s="84"/>
+      <c r="E28" s="84"/>
+      <c r="F28" s="84"/>
+      <c r="G28" s="84"/>
+      <c r="H28" s="84"/>
+      <c r="I28" s="21">
         <v>41153</v>
       </c>
-      <c r="J28" s="24">
+      <c r="J28" s="93">
         <v>41306</v>
       </c>
       <c r="K28" s="6">
         <v>41426</v>
       </c>
-      <c r="L28" s="57"/>
-      <c r="M28" s="57"/>
-      <c r="N28" s="57"/>
-      <c r="O28" s="68"/>
-      <c r="P28" s="81"/>
+      <c r="L28" s="74"/>
+      <c r="M28" s="74"/>
+      <c r="N28" s="74"/>
+      <c r="O28" s="65"/>
+      <c r="P28" s="48"/>
     </row>
     <row r="29" spans="1:16" ht="15.5">
-      <c r="A29" s="46"/>
-      <c r="B29" s="46">
+      <c r="A29" s="83"/>
+      <c r="B29" s="83">
         <v>1</v>
       </c>
-      <c r="C29" s="46" t="s">
+      <c r="C29" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="83" t="s">
         <v>49</v>
       </c>
-      <c r="E29" s="46" t="s">
+      <c r="E29" s="83" t="s">
         <v>50</v>
       </c>
-      <c r="F29" s="46" t="s">
+      <c r="F29" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G29" s="46" t="s">
+      <c r="G29" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="H29" s="46" t="s">
+      <c r="H29" s="83" t="s">
         <v>51</v>
       </c>
       <c r="I29" s="2">
         <v>40817</v>
       </c>
-      <c r="J29" s="25">
+      <c r="J29" s="24">
         <v>41000</v>
       </c>
-      <c r="K29" s="18">
+      <c r="K29" s="17">
         <v>41365</v>
       </c>
-      <c r="L29" s="57">
+      <c r="L29" s="74">
         <v>246698</v>
       </c>
-      <c r="M29" s="57">
+      <c r="M29" s="74">
         <v>0</v>
       </c>
-      <c r="N29" s="57">
+      <c r="N29" s="74">
         <v>280988</v>
       </c>
-      <c r="O29" s="68">
+      <c r="O29" s="65">
         <v>0.3</v>
       </c>
-      <c r="P29" s="81">
+      <c r="P29" s="48">
         <v>527686</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="15.5">
-      <c r="A30" s="47"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="47"/>
-      <c r="G30" s="47"/>
-      <c r="H30" s="47"/>
-      <c r="I30" s="26">
+      <c r="A30" s="84"/>
+      <c r="B30" s="84"/>
+      <c r="C30" s="84"/>
+      <c r="D30" s="84"/>
+      <c r="E30" s="84"/>
+      <c r="F30" s="84"/>
+      <c r="G30" s="84"/>
+      <c r="H30" s="84"/>
+      <c r="I30" s="25">
         <v>40817</v>
       </c>
-      <c r="J30" s="26">
+      <c r="J30" s="25">
         <v>41000</v>
       </c>
-      <c r="K30" s="24">
+      <c r="K30" s="23">
         <v>41365</v>
       </c>
-      <c r="L30" s="57"/>
-      <c r="M30" s="57"/>
-      <c r="N30" s="57"/>
-      <c r="O30" s="68"/>
-      <c r="P30" s="81"/>
+      <c r="L30" s="74"/>
+      <c r="M30" s="74"/>
+      <c r="N30" s="74"/>
+      <c r="O30" s="65"/>
+      <c r="P30" s="48"/>
     </row>
     <row r="31" spans="1:16" ht="15.5">
-      <c r="A31" s="46"/>
-      <c r="B31" s="46">
+      <c r="A31" s="83"/>
+      <c r="B31" s="83">
         <v>1</v>
       </c>
-      <c r="C31" s="46" t="s">
+      <c r="C31" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="46" t="s">
+      <c r="D31" s="83" t="s">
         <v>52</v>
       </c>
-      <c r="E31" s="46" t="s">
+      <c r="E31" s="83" t="s">
         <v>53</v>
       </c>
-      <c r="F31" s="46" t="s">
+      <c r="F31" s="83" t="s">
         <v>54</v>
       </c>
-      <c r="G31" s="53" t="s">
+      <c r="G31" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="H31" s="46" t="s">
+      <c r="H31" s="83" t="s">
         <v>56</v>
       </c>
       <c r="I31" s="2">
         <v>41183</v>
       </c>
-      <c r="J31" s="25">
+      <c r="J31" s="24">
         <v>41760</v>
       </c>
-      <c r="K31" s="18">
+      <c r="K31" s="17">
         <v>41609</v>
       </c>
-      <c r="L31" s="55">
+      <c r="L31" s="53">
         <v>0</v>
       </c>
-      <c r="M31" s="55">
+      <c r="M31" s="53">
         <v>0</v>
       </c>
-      <c r="N31" s="55">
+      <c r="N31" s="53">
         <v>151470</v>
       </c>
-      <c r="O31" s="69">
+      <c r="O31" s="66">
         <v>0.3</v>
       </c>
-      <c r="P31" s="81">
+      <c r="P31" s="48">
         <v>151470</v>
       </c>
     </row>
     <row r="32" spans="1:16" ht="15.5">
-      <c r="A32" s="47"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="54"/>
-      <c r="H32" s="47"/>
+      <c r="A32" s="84"/>
+      <c r="B32" s="84"/>
+      <c r="C32" s="84"/>
+      <c r="D32" s="84"/>
+      <c r="E32" s="84"/>
+      <c r="F32" s="84"/>
+      <c r="G32" s="79"/>
+      <c r="H32" s="84"/>
       <c r="I32" s="8">
         <v>41183</v>
       </c>
@@ -2576,72 +2588,72 @@
       <c r="K32" s="6">
         <v>41609</v>
       </c>
-      <c r="L32" s="56"/>
-      <c r="M32" s="56"/>
-      <c r="N32" s="56"/>
-      <c r="O32" s="70"/>
-      <c r="P32" s="81"/>
+      <c r="L32" s="54"/>
+      <c r="M32" s="54"/>
+      <c r="N32" s="54"/>
+      <c r="O32" s="67"/>
+      <c r="P32" s="48"/>
     </row>
     <row r="33" spans="1:16" ht="15.5">
-      <c r="A33" s="46">
+      <c r="A33" s="83">
         <v>2</v>
       </c>
-      <c r="B33" s="46">
+      <c r="B33" s="83">
         <v>2</v>
       </c>
-      <c r="C33" s="46" t="s">
+      <c r="C33" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="46" t="s">
+      <c r="D33" s="83" t="s">
         <v>57</v>
       </c>
-      <c r="E33" s="46" t="s">
+      <c r="E33" s="83" t="s">
         <v>58</v>
       </c>
-      <c r="F33" s="46" t="s">
+      <c r="F33" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G33" s="46" t="s">
+      <c r="G33" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="H33" s="46" t="s">
+      <c r="H33" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="I33" s="20">
+      <c r="I33" s="19">
         <v>41365</v>
       </c>
-      <c r="J33" s="25">
+      <c r="J33" s="24">
         <v>41579</v>
       </c>
-      <c r="K33" s="25">
+      <c r="K33" s="24">
         <v>41579</v>
       </c>
-      <c r="L33" s="55">
+      <c r="L33" s="53">
         <v>150000</v>
       </c>
-      <c r="M33" s="55">
+      <c r="M33" s="53">
         <v>0</v>
       </c>
-      <c r="N33" s="55">
+      <c r="N33" s="53">
         <v>0</v>
       </c>
-      <c r="O33" s="69">
+      <c r="O33" s="66">
         <v>0.5</v>
       </c>
-      <c r="P33" s="81">
+      <c r="P33" s="48">
         <v>150000</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="15.5">
-      <c r="A34" s="47"/>
-      <c r="B34" s="47"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="22">
+      <c r="A34" s="84"/>
+      <c r="B34" s="84"/>
+      <c r="C34" s="84"/>
+      <c r="D34" s="84"/>
+      <c r="E34" s="84"/>
+      <c r="F34" s="84"/>
+      <c r="G34" s="84"/>
+      <c r="H34" s="84"/>
+      <c r="I34" s="21">
         <v>41365</v>
       </c>
       <c r="J34" s="5">
@@ -2650,72 +2662,72 @@
       <c r="K34" s="5">
         <v>41579</v>
       </c>
-      <c r="L34" s="56"/>
-      <c r="M34" s="56"/>
-      <c r="N34" s="56"/>
-      <c r="O34" s="70"/>
-      <c r="P34" s="81"/>
+      <c r="L34" s="54"/>
+      <c r="M34" s="54"/>
+      <c r="N34" s="54"/>
+      <c r="O34" s="67"/>
+      <c r="P34" s="48"/>
     </row>
     <row r="35" spans="1:16" ht="15.5">
-      <c r="A35" s="46">
+      <c r="A35" s="83">
         <v>2</v>
       </c>
-      <c r="B35" s="46">
+      <c r="B35" s="83">
         <v>2</v>
       </c>
-      <c r="C35" s="46" t="s">
+      <c r="C35" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="46" t="s">
+      <c r="D35" s="83" t="s">
         <v>59</v>
       </c>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="F35" s="46" t="s">
+      <c r="F35" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G35" s="46" t="s">
+      <c r="G35" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="H35" s="46" t="s">
+      <c r="H35" s="83" t="s">
         <v>61</v>
       </c>
       <c r="I35" s="2">
         <v>41306</v>
       </c>
-      <c r="J35" s="18">
+      <c r="J35" s="17">
         <v>41699</v>
       </c>
-      <c r="K35" s="18">
+      <c r="K35" s="17">
         <v>41579</v>
       </c>
-      <c r="L35" s="58">
+      <c r="L35" s="75">
         <v>76880</v>
       </c>
-      <c r="M35" s="58">
+      <c r="M35" s="75">
         <v>206000</v>
       </c>
-      <c r="N35" s="58">
+      <c r="N35" s="75">
         <v>0</v>
       </c>
-      <c r="O35" s="71">
+      <c r="O35" s="68">
         <v>0.5</v>
       </c>
-      <c r="P35" s="82">
+      <c r="P35" s="55">
         <v>282880</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="15.5">
-      <c r="A36" s="47"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="47"/>
-      <c r="F36" s="47"/>
-      <c r="G36" s="47"/>
-      <c r="H36" s="47"/>
-      <c r="I36" s="26">
+      <c r="A36" s="84"/>
+      <c r="B36" s="84"/>
+      <c r="C36" s="84"/>
+      <c r="D36" s="84"/>
+      <c r="E36" s="84"/>
+      <c r="F36" s="84"/>
+      <c r="G36" s="84"/>
+      <c r="H36" s="84"/>
+      <c r="I36" s="25">
         <v>41306</v>
       </c>
       <c r="J36" s="6">
@@ -2724,72 +2736,72 @@
       <c r="K36" s="6">
         <v>41579</v>
       </c>
-      <c r="L36" s="59"/>
-      <c r="M36" s="59"/>
-      <c r="N36" s="59"/>
-      <c r="O36" s="72"/>
-      <c r="P36" s="83"/>
+      <c r="L36" s="76"/>
+      <c r="M36" s="76"/>
+      <c r="N36" s="76"/>
+      <c r="O36" s="69"/>
+      <c r="P36" s="56"/>
     </row>
     <row r="37" spans="1:16" ht="15.5">
-      <c r="A37" s="46">
+      <c r="A37" s="83">
         <v>2</v>
       </c>
-      <c r="B37" s="46">
+      <c r="B37" s="83">
         <v>2</v>
       </c>
-      <c r="C37" s="46" t="s">
+      <c r="C37" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="D37" s="46" t="s">
+      <c r="D37" s="83" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="46" t="s">
+      <c r="E37" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="F37" s="46" t="s">
+      <c r="F37" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="G37" s="46" t="s">
+      <c r="G37" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="H37" s="46" t="s">
+      <c r="H37" s="83" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="2">
         <v>41334</v>
       </c>
-      <c r="J37" s="25">
+      <c r="J37" s="24">
         <v>41518</v>
       </c>
-      <c r="K37" s="18">
+      <c r="K37" s="17">
         <v>41518</v>
       </c>
-      <c r="L37" s="57">
+      <c r="L37" s="74">
         <v>141750</v>
       </c>
-      <c r="M37" s="57">
+      <c r="M37" s="74">
         <v>0</v>
       </c>
-      <c r="N37" s="57">
+      <c r="N37" s="74">
         <v>121500</v>
       </c>
-      <c r="O37" s="68">
+      <c r="O37" s="65">
         <v>0.75</v>
       </c>
-      <c r="P37" s="81">
+      <c r="P37" s="48">
         <v>263250</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="15.5">
-      <c r="A38" s="47"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="26">
+      <c r="A38" s="84"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="84"/>
+      <c r="D38" s="84"/>
+      <c r="E38" s="84"/>
+      <c r="F38" s="84"/>
+      <c r="G38" s="84"/>
+      <c r="H38" s="84"/>
+      <c r="I38" s="25">
         <v>41334</v>
       </c>
       <c r="J38" s="5">
@@ -2798,35 +2810,35 @@
       <c r="K38" s="6">
         <v>41518</v>
       </c>
-      <c r="L38" s="57"/>
-      <c r="M38" s="57"/>
-      <c r="N38" s="57"/>
-      <c r="O38" s="68"/>
-      <c r="P38" s="81"/>
+      <c r="L38" s="74"/>
+      <c r="M38" s="74"/>
+      <c r="N38" s="74"/>
+      <c r="O38" s="65"/>
+      <c r="P38" s="48"/>
     </row>
     <row r="39" spans="1:16" ht="15.5">
-      <c r="A39" s="48">
+      <c r="A39" s="85">
         <v>1</v>
       </c>
-      <c r="B39" s="45">
+      <c r="B39" s="77">
         <v>1</v>
       </c>
-      <c r="C39" s="46" t="s">
+      <c r="C39" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="D39" s="45" t="s">
+      <c r="D39" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="E39" s="45" t="s">
+      <c r="E39" s="77" t="s">
         <v>67</v>
       </c>
-      <c r="F39" s="45" t="s">
+      <c r="F39" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="G39" s="45" t="s">
+      <c r="G39" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="H39" s="45" t="s">
+      <c r="H39" s="77" t="s">
         <v>40</v>
       </c>
       <c r="I39" s="2">
@@ -2838,65 +2850,65 @@
       <c r="K39" s="14">
         <v>41426</v>
       </c>
-      <c r="L39" s="60">
+      <c r="L39" s="72">
         <v>347200</v>
       </c>
-      <c r="M39" s="60">
+      <c r="M39" s="72">
         <v>644800</v>
       </c>
-      <c r="N39" s="60">
+      <c r="N39" s="72">
         <v>0</v>
       </c>
-      <c r="O39" s="73">
+      <c r="O39" s="59">
         <v>0.75</v>
       </c>
-      <c r="P39" s="81">
+      <c r="P39" s="48">
         <v>992000</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="15.5">
-      <c r="A40" s="48"/>
-      <c r="B40" s="45"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="21">
+      <c r="A40" s="85"/>
+      <c r="B40" s="77"/>
+      <c r="C40" s="84"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
+      <c r="G40" s="77"/>
+      <c r="H40" s="77"/>
+      <c r="I40" s="20">
         <v>41275</v>
       </c>
       <c r="J40" s="11"/>
       <c r="K40" s="6"/>
-      <c r="L40" s="60"/>
-      <c r="M40" s="60"/>
-      <c r="N40" s="60"/>
-      <c r="O40" s="73"/>
-      <c r="P40" s="81"/>
+      <c r="L40" s="72"/>
+      <c r="M40" s="72"/>
+      <c r="N40" s="72"/>
+      <c r="O40" s="59"/>
+      <c r="P40" s="48"/>
     </row>
     <row r="41" spans="1:16" ht="15.5">
-      <c r="A41" s="48">
+      <c r="A41" s="85">
         <v>1</v>
       </c>
-      <c r="B41" s="45">
+      <c r="B41" s="77">
         <v>1</v>
       </c>
-      <c r="C41" s="46" t="s">
+      <c r="C41" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="D41" s="45" t="s">
+      <c r="D41" s="77" t="s">
         <v>69</v>
       </c>
-      <c r="E41" s="45" t="s">
+      <c r="E41" s="77" t="s">
         <v>70</v>
       </c>
-      <c r="F41" s="45" t="s">
+      <c r="F41" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G41" s="45" t="s">
+      <c r="G41" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="H41" s="45" t="s">
+      <c r="H41" s="77" t="s">
         <v>71</v>
       </c>
       <c r="I41" s="2">
@@ -2908,271 +2920,271 @@
       <c r="K41" s="2">
         <v>41334</v>
       </c>
-      <c r="L41" s="61">
+      <c r="L41" s="73">
         <v>200000</v>
       </c>
-      <c r="M41" s="61">
+      <c r="M41" s="73">
         <v>0</v>
       </c>
-      <c r="N41" s="61">
+      <c r="N41" s="73">
         <v>0</v>
       </c>
-      <c r="O41" s="74">
+      <c r="O41" s="60">
         <v>0.8</v>
       </c>
-      <c r="P41" s="81">
+      <c r="P41" s="48">
         <v>200000</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="15.5">
-      <c r="A42" s="48"/>
-      <c r="B42" s="45"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="45"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="45"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="21">
+      <c r="A42" s="85"/>
+      <c r="B42" s="77"/>
+      <c r="C42" s="84"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
+      <c r="I42" s="20">
         <v>41153</v>
       </c>
-      <c r="J42" s="21">
+      <c r="J42" s="20">
         <v>41244</v>
       </c>
-      <c r="K42" s="24">
+      <c r="K42" s="93">
         <v>41396</v>
       </c>
-      <c r="L42" s="61"/>
-      <c r="M42" s="61"/>
-      <c r="N42" s="61"/>
-      <c r="O42" s="74"/>
-      <c r="P42" s="81"/>
+      <c r="L42" s="73"/>
+      <c r="M42" s="73"/>
+      <c r="N42" s="73"/>
+      <c r="O42" s="60"/>
+      <c r="P42" s="48"/>
     </row>
     <row r="43" spans="1:16" ht="15.5">
-      <c r="A43" s="49">
+      <c r="A43" s="86">
         <v>1</v>
       </c>
-      <c r="B43" s="50">
+      <c r="B43" s="80">
         <v>2</v>
       </c>
-      <c r="C43" s="51" t="s">
+      <c r="C43" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D43" s="50" t="s">
+      <c r="D43" s="80" t="s">
         <v>73</v>
       </c>
-      <c r="E43" s="50" t="s">
+      <c r="E43" s="80" t="s">
         <v>74</v>
       </c>
-      <c r="F43" s="50" t="s">
+      <c r="F43" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="G43" s="50" t="s">
+      <c r="G43" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="H43" s="50">
+      <c r="H43" s="80">
         <v>737</v>
       </c>
-      <c r="I43" s="27">
+      <c r="I43" s="26">
         <v>41334</v>
       </c>
-      <c r="J43" s="27">
+      <c r="J43" s="26">
         <v>41821</v>
       </c>
-      <c r="K43" s="28">
+      <c r="K43" s="27">
         <v>41883</v>
       </c>
-      <c r="L43" s="62">
+      <c r="L43" s="70">
         <v>250800</v>
       </c>
-      <c r="M43" s="62">
+      <c r="M43" s="70">
         <v>0</v>
       </c>
-      <c r="N43" s="62">
+      <c r="N43" s="70">
         <v>38760</v>
       </c>
-      <c r="O43" s="75">
+      <c r="O43" s="57">
         <v>0.5</v>
       </c>
-      <c r="P43" s="84">
+      <c r="P43" s="45">
         <v>289560</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="15.5">
-      <c r="A44" s="49"/>
-      <c r="B44" s="50"/>
-      <c r="C44" s="52"/>
-      <c r="D44" s="50"/>
-      <c r="E44" s="50"/>
-      <c r="F44" s="50"/>
-      <c r="G44" s="50"/>
-      <c r="H44" s="50"/>
-      <c r="I44" s="29">
+      <c r="A44" s="86"/>
+      <c r="B44" s="80"/>
+      <c r="C44" s="82"/>
+      <c r="D44" s="80"/>
+      <c r="E44" s="80"/>
+      <c r="F44" s="80"/>
+      <c r="G44" s="80"/>
+      <c r="H44" s="80"/>
+      <c r="I44" s="28">
         <v>41334</v>
       </c>
-      <c r="J44" s="30"/>
-      <c r="K44" s="31"/>
-      <c r="L44" s="62"/>
-      <c r="M44" s="62"/>
-      <c r="N44" s="62"/>
-      <c r="O44" s="75"/>
-      <c r="P44" s="84"/>
+      <c r="J44" s="29"/>
+      <c r="K44" s="30"/>
+      <c r="L44" s="70"/>
+      <c r="M44" s="70"/>
+      <c r="N44" s="70"/>
+      <c r="O44" s="57"/>
+      <c r="P44" s="45"/>
     </row>
     <row r="45" spans="1:16" ht="15.5">
-      <c r="A45" s="49">
+      <c r="A45" s="86">
         <v>1</v>
       </c>
-      <c r="B45" s="50">
+      <c r="B45" s="80">
         <v>2</v>
       </c>
-      <c r="C45" s="51" t="s">
+      <c r="C45" s="81" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="50" t="s">
+      <c r="D45" s="80" t="s">
         <v>75</v>
       </c>
-      <c r="E45" s="50" t="s">
+      <c r="E45" s="80" t="s">
         <v>76</v>
       </c>
-      <c r="F45" s="50" t="s">
+      <c r="F45" s="80" t="s">
         <v>68</v>
       </c>
-      <c r="G45" s="50" t="s">
+      <c r="G45" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="H45" s="50" t="s">
+      <c r="H45" s="80" t="s">
         <v>77</v>
       </c>
-      <c r="I45" s="27">
+      <c r="I45" s="26">
         <v>41395</v>
       </c>
-      <c r="J45" s="27">
+      <c r="J45" s="26">
         <v>41518</v>
       </c>
-      <c r="K45" s="28">
+      <c r="K45" s="27">
         <v>41640</v>
       </c>
-      <c r="L45" s="62"/>
-      <c r="M45" s="62"/>
-      <c r="N45" s="62"/>
-      <c r="O45" s="75">
+      <c r="L45" s="70"/>
+      <c r="M45" s="70"/>
+      <c r="N45" s="70"/>
+      <c r="O45" s="57">
         <v>0.75</v>
       </c>
-      <c r="P45" s="84"/>
+      <c r="P45" s="45"/>
     </row>
     <row r="46" spans="1:16" ht="15.5">
-      <c r="A46" s="49"/>
-      <c r="B46" s="50"/>
-      <c r="C46" s="52"/>
-      <c r="D46" s="50"/>
-      <c r="E46" s="50"/>
-      <c r="F46" s="50"/>
-      <c r="G46" s="50"/>
-      <c r="H46" s="50"/>
-      <c r="I46" s="32"/>
-      <c r="J46" s="30"/>
-      <c r="K46" s="31"/>
-      <c r="L46" s="62"/>
-      <c r="M46" s="62"/>
-      <c r="N46" s="62"/>
-      <c r="O46" s="75"/>
-      <c r="P46" s="84"/>
+      <c r="A46" s="86"/>
+      <c r="B46" s="80"/>
+      <c r="C46" s="82"/>
+      <c r="D46" s="80"/>
+      <c r="E46" s="80"/>
+      <c r="F46" s="80"/>
+      <c r="G46" s="80"/>
+      <c r="H46" s="80"/>
+      <c r="I46" s="31"/>
+      <c r="J46" s="29"/>
+      <c r="K46" s="30"/>
+      <c r="L46" s="70"/>
+      <c r="M46" s="70"/>
+      <c r="N46" s="70"/>
+      <c r="O46" s="57"/>
+      <c r="P46" s="45"/>
     </row>
     <row r="47" spans="1:16" ht="15.5">
-      <c r="A47" s="50">
+      <c r="A47" s="80">
         <v>2</v>
       </c>
-      <c r="B47" s="50">
+      <c r="B47" s="80">
         <v>1</v>
       </c>
-      <c r="C47" s="51" t="s">
+      <c r="C47" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D47" s="50" t="s">
+      <c r="D47" s="80" t="s">
         <v>78</v>
       </c>
-      <c r="E47" s="50" t="s">
+      <c r="E47" s="80" t="s">
         <v>79</v>
       </c>
-      <c r="F47" s="50" t="s">
+      <c r="F47" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="G47" s="50" t="s">
+      <c r="G47" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="H47" s="50" t="s">
+      <c r="H47" s="80" t="s">
         <v>80</v>
       </c>
-      <c r="I47" s="27">
+      <c r="I47" s="26">
         <v>41061</v>
       </c>
-      <c r="J47" s="27" t="s">
+      <c r="J47" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="K47" s="28">
+      <c r="K47" s="27">
         <v>41426</v>
       </c>
-      <c r="L47" s="63">
+      <c r="L47" s="71">
         <v>43400</v>
       </c>
-      <c r="M47" s="63">
+      <c r="M47" s="71">
         <v>0</v>
       </c>
-      <c r="N47" s="63">
+      <c r="N47" s="71">
         <v>69720</v>
       </c>
-      <c r="O47" s="76">
+      <c r="O47" s="58">
         <v>0.33</v>
       </c>
-      <c r="P47" s="84">
+      <c r="P47" s="45">
         <v>113120</v>
       </c>
     </row>
     <row r="48" spans="1:16" ht="15.5">
-      <c r="A48" s="50"/>
-      <c r="B48" s="50"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="50"/>
-      <c r="E48" s="50"/>
-      <c r="F48" s="50"/>
-      <c r="G48" s="50"/>
-      <c r="H48" s="50"/>
-      <c r="I48" s="29">
+      <c r="A48" s="80"/>
+      <c r="B48" s="80"/>
+      <c r="C48" s="82"/>
+      <c r="D48" s="80"/>
+      <c r="E48" s="80"/>
+      <c r="F48" s="80"/>
+      <c r="G48" s="80"/>
+      <c r="H48" s="80"/>
+      <c r="I48" s="28">
         <v>41061</v>
       </c>
-      <c r="J48" s="33">
+      <c r="J48" s="94">
         <v>41275</v>
       </c>
-      <c r="K48" s="34"/>
-      <c r="L48" s="63"/>
-      <c r="M48" s="63"/>
-      <c r="N48" s="63"/>
-      <c r="O48" s="76"/>
-      <c r="P48" s="84"/>
+      <c r="K48" s="32"/>
+      <c r="L48" s="71"/>
+      <c r="M48" s="71"/>
+      <c r="N48" s="71"/>
+      <c r="O48" s="58"/>
+      <c r="P48" s="45"/>
     </row>
     <row r="49" spans="1:16" ht="15.5">
-      <c r="A49" s="45">
+      <c r="A49" s="77">
         <v>2</v>
       </c>
-      <c r="B49" s="45">
+      <c r="B49" s="77">
         <v>1</v>
       </c>
-      <c r="C49" s="46" t="s">
+      <c r="C49" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="D49" s="45" t="s">
+      <c r="D49" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="E49" s="45" t="s">
+      <c r="E49" s="77" t="s">
         <v>67</v>
       </c>
-      <c r="F49" s="45" t="s">
+      <c r="F49" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G49" s="45" t="s">
+      <c r="G49" s="77" t="s">
         <v>82</v>
       </c>
-      <c r="H49" s="53" t="s">
+      <c r="H49" s="78" t="s">
         <v>40</v>
       </c>
       <c r="I49" s="2">
@@ -3184,135 +3196,135 @@
       <c r="K49" s="14">
         <v>41609</v>
       </c>
-      <c r="L49" s="60">
+      <c r="L49" s="72">
         <v>0</v>
       </c>
-      <c r="M49" s="60">
+      <c r="M49" s="72">
         <v>0</v>
       </c>
-      <c r="N49" s="60">
+      <c r="N49" s="72">
         <v>108500</v>
       </c>
-      <c r="O49" s="73">
+      <c r="O49" s="59">
         <v>0.75</v>
       </c>
-      <c r="P49" s="81">
+      <c r="P49" s="48">
         <v>108500</v>
       </c>
     </row>
     <row r="50" spans="1:16" ht="15.5">
-      <c r="A50" s="45"/>
-      <c r="B50" s="45"/>
-      <c r="C50" s="47"/>
-      <c r="D50" s="45"/>
-      <c r="E50" s="45"/>
-      <c r="F50" s="45"/>
-      <c r="G50" s="45"/>
-      <c r="H50" s="54"/>
-      <c r="I50" s="21">
+      <c r="A50" s="77"/>
+      <c r="B50" s="77"/>
+      <c r="C50" s="84"/>
+      <c r="D50" s="77"/>
+      <c r="E50" s="77"/>
+      <c r="F50" s="77"/>
+      <c r="G50" s="77"/>
+      <c r="H50" s="79"/>
+      <c r="I50" s="20">
         <v>41061</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="6"/>
-      <c r="L50" s="60"/>
-      <c r="M50" s="60"/>
-      <c r="N50" s="60"/>
-      <c r="O50" s="73"/>
-      <c r="P50" s="81"/>
+      <c r="L50" s="72"/>
+      <c r="M50" s="72"/>
+      <c r="N50" s="72"/>
+      <c r="O50" s="59"/>
+      <c r="P50" s="48"/>
     </row>
     <row r="51" spans="1:16" ht="15.5">
-      <c r="A51" s="50">
+      <c r="A51" s="80">
         <v>2</v>
       </c>
-      <c r="B51" s="50">
+      <c r="B51" s="80">
         <v>1</v>
       </c>
-      <c r="C51" s="51" t="s">
+      <c r="C51" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D51" s="50" t="s">
+      <c r="D51" s="80" t="s">
         <v>83</v>
       </c>
-      <c r="E51" s="50" t="s">
+      <c r="E51" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="F51" s="50" t="s">
+      <c r="F51" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="G51" s="50" t="s">
+      <c r="G51" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="H51" s="50">
+      <c r="H51" s="80">
         <v>737</v>
       </c>
-      <c r="I51" s="27">
+      <c r="I51" s="26">
         <v>41334</v>
       </c>
       <c r="J51" s="2">
         <v>41699</v>
       </c>
-      <c r="K51" s="28">
+      <c r="K51" s="27">
         <v>41791</v>
       </c>
-      <c r="L51" s="63">
+      <c r="L51" s="71">
         <v>501600</v>
       </c>
-      <c r="M51" s="63">
+      <c r="M51" s="71">
         <v>0</v>
       </c>
-      <c r="N51" s="63">
+      <c r="N51" s="71">
         <v>77520</v>
       </c>
-      <c r="O51" s="76">
+      <c r="O51" s="58">
         <v>0.33</v>
       </c>
-      <c r="P51" s="84">
+      <c r="P51" s="45">
         <v>579120</v>
       </c>
     </row>
     <row r="52" spans="1:16" ht="15.5">
-      <c r="A52" s="50"/>
-      <c r="B52" s="50"/>
-      <c r="C52" s="52"/>
-      <c r="D52" s="50"/>
-      <c r="E52" s="50"/>
-      <c r="F52" s="50"/>
-      <c r="G52" s="50"/>
-      <c r="H52" s="50"/>
-      <c r="I52" s="29">
+      <c r="A52" s="80"/>
+      <c r="B52" s="80"/>
+      <c r="C52" s="82"/>
+      <c r="D52" s="80"/>
+      <c r="E52" s="80"/>
+      <c r="F52" s="80"/>
+      <c r="G52" s="80"/>
+      <c r="H52" s="80"/>
+      <c r="I52" s="28">
         <v>41334</v>
       </c>
-      <c r="J52" s="32"/>
-      <c r="K52" s="34"/>
-      <c r="L52" s="63"/>
-      <c r="M52" s="63"/>
-      <c r="N52" s="63"/>
-      <c r="O52" s="76"/>
-      <c r="P52" s="84"/>
+      <c r="J52" s="31"/>
+      <c r="K52" s="32"/>
+      <c r="L52" s="71"/>
+      <c r="M52" s="71"/>
+      <c r="N52" s="71"/>
+      <c r="O52" s="58"/>
+      <c r="P52" s="45"/>
     </row>
     <row r="53" spans="1:16" ht="15.5">
-      <c r="A53" s="45">
+      <c r="A53" s="77">
         <v>2</v>
       </c>
-      <c r="B53" s="45">
+      <c r="B53" s="77">
         <v>2</v>
       </c>
-      <c r="C53" s="46" t="s">
+      <c r="C53" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="D53" s="45" t="s">
+      <c r="D53" s="77" t="s">
         <v>85</v>
       </c>
-      <c r="E53" s="45" t="s">
+      <c r="E53" s="77" t="s">
         <v>86</v>
       </c>
-      <c r="F53" s="45" t="s">
+      <c r="F53" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="G53" s="45" t="s">
+      <c r="G53" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="H53" s="45">
+      <c r="H53" s="77">
         <v>737</v>
       </c>
       <c r="I53" s="2">
@@ -3324,65 +3336,65 @@
       <c r="K53" s="14">
         <v>41760</v>
       </c>
-      <c r="L53" s="61">
+      <c r="L53" s="73">
         <v>2503600</v>
       </c>
-      <c r="M53" s="61">
+      <c r="M53" s="73">
         <v>0</v>
       </c>
-      <c r="N53" s="61">
+      <c r="N53" s="73">
         <v>128973.33333333299</v>
       </c>
-      <c r="O53" s="74">
+      <c r="O53" s="60">
         <v>0.5</v>
       </c>
-      <c r="P53" s="81">
+      <c r="P53" s="48">
         <v>2632573.3333333302</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="15.5">
-      <c r="A54" s="45"/>
-      <c r="B54" s="45"/>
-      <c r="C54" s="47"/>
-      <c r="D54" s="45"/>
-      <c r="E54" s="45"/>
-      <c r="F54" s="45"/>
-      <c r="G54" s="45"/>
-      <c r="H54" s="45"/>
-      <c r="I54" s="21">
+      <c r="A54" s="77"/>
+      <c r="B54" s="77"/>
+      <c r="C54" s="84"/>
+      <c r="D54" s="77"/>
+      <c r="E54" s="77"/>
+      <c r="F54" s="77"/>
+      <c r="G54" s="77"/>
+      <c r="H54" s="77"/>
+      <c r="I54" s="20">
         <v>41275</v>
       </c>
-      <c r="J54" s="35"/>
+      <c r="J54" s="33"/>
       <c r="K54" s="6"/>
-      <c r="L54" s="61"/>
-      <c r="M54" s="61"/>
-      <c r="N54" s="61"/>
-      <c r="O54" s="74"/>
-      <c r="P54" s="81"/>
+      <c r="L54" s="73"/>
+      <c r="M54" s="73"/>
+      <c r="N54" s="73"/>
+      <c r="O54" s="60"/>
+      <c r="P54" s="48"/>
     </row>
     <row r="55" spans="1:16" ht="15.5">
-      <c r="A55" s="45">
+      <c r="A55" s="77">
         <v>2</v>
       </c>
-      <c r="B55" s="45">
+      <c r="B55" s="77">
         <v>2</v>
       </c>
-      <c r="C55" s="46" t="s">
+      <c r="C55" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="D55" s="45" t="s">
+      <c r="D55" s="77" t="s">
         <v>87</v>
       </c>
-      <c r="E55" s="45" t="s">
+      <c r="E55" s="77" t="s">
         <v>88</v>
       </c>
-      <c r="F55" s="45" t="s">
+      <c r="F55" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G55" s="45" t="s">
+      <c r="G55" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="H55" s="53" t="s">
+      <c r="H55" s="78" t="s">
         <v>40</v>
       </c>
       <c r="I55" s="2">
@@ -3394,571 +3406,963 @@
       <c r="K55" s="2">
         <v>41548</v>
       </c>
-      <c r="L55" s="61">
+      <c r="L55" s="73">
         <v>268800</v>
       </c>
-      <c r="M55" s="61">
+      <c r="M55" s="73">
         <v>499200</v>
       </c>
-      <c r="N55" s="61">
+      <c r="N55" s="73">
         <v>0</v>
       </c>
-      <c r="O55" s="74">
+      <c r="O55" s="60">
         <v>0.6</v>
       </c>
-      <c r="P55" s="81">
+      <c r="P55" s="48">
         <v>768000</v>
       </c>
     </row>
     <row r="56" spans="1:16" ht="15.5">
-      <c r="A56" s="45"/>
-      <c r="B56" s="45"/>
-      <c r="C56" s="47"/>
-      <c r="D56" s="45"/>
-      <c r="E56" s="45"/>
-      <c r="F56" s="45"/>
-      <c r="G56" s="45"/>
-      <c r="H56" s="54"/>
-      <c r="I56" s="21">
+      <c r="A56" s="77"/>
+      <c r="B56" s="77"/>
+      <c r="C56" s="84"/>
+      <c r="D56" s="77"/>
+      <c r="E56" s="77"/>
+      <c r="F56" s="77"/>
+      <c r="G56" s="77"/>
+      <c r="H56" s="79"/>
+      <c r="I56" s="20">
         <v>41153</v>
       </c>
       <c r="J56" s="6"/>
       <c r="K56" s="6"/>
-      <c r="L56" s="61"/>
-      <c r="M56" s="61"/>
-      <c r="N56" s="61"/>
-      <c r="O56" s="74"/>
-      <c r="P56" s="81"/>
+      <c r="L56" s="73"/>
+      <c r="M56" s="73"/>
+      <c r="N56" s="73"/>
+      <c r="O56" s="60"/>
+      <c r="P56" s="48"/>
     </row>
     <row r="57" spans="1:16" ht="15.5">
-      <c r="A57" s="50">
+      <c r="A57" s="80">
         <v>3</v>
       </c>
-      <c r="B57" s="50">
+      <c r="B57" s="80">
         <v>2</v>
       </c>
-      <c r="C57" s="51" t="s">
+      <c r="C57" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D57" s="50" t="s">
+      <c r="D57" s="80" t="s">
         <v>78</v>
       </c>
-      <c r="E57" s="50" t="s">
+      <c r="E57" s="80" t="s">
         <v>79</v>
       </c>
-      <c r="F57" s="50" t="s">
+      <c r="F57" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="G57" s="50" t="s">
+      <c r="G57" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="H57" s="50">
+      <c r="H57" s="80">
         <v>737</v>
       </c>
-      <c r="I57" s="27">
+      <c r="I57" s="26">
         <v>41061</v>
       </c>
-      <c r="J57" s="27">
+      <c r="J57" s="26">
         <v>41426</v>
       </c>
-      <c r="K57" s="28">
+      <c r="K57" s="27">
         <v>41426</v>
       </c>
-      <c r="L57" s="63">
+      <c r="L57" s="71">
         <v>198000</v>
       </c>
-      <c r="M57" s="63">
+      <c r="M57" s="71">
         <v>0</v>
       </c>
-      <c r="N57" s="63">
+      <c r="N57" s="71">
         <v>61200</v>
       </c>
-      <c r="O57" s="76">
+      <c r="O57" s="58">
         <v>0.33</v>
       </c>
-      <c r="P57" s="84">
+      <c r="P57" s="45">
         <v>259200</v>
       </c>
     </row>
     <row r="58" spans="1:16" ht="15.5">
-      <c r="A58" s="50"/>
-      <c r="B58" s="50"/>
-      <c r="C58" s="52"/>
-      <c r="D58" s="50"/>
-      <c r="E58" s="50"/>
-      <c r="F58" s="50"/>
-      <c r="G58" s="50"/>
-      <c r="H58" s="50"/>
-      <c r="I58" s="29">
+      <c r="A58" s="80"/>
+      <c r="B58" s="80"/>
+      <c r="C58" s="82"/>
+      <c r="D58" s="80"/>
+      <c r="E58" s="80"/>
+      <c r="F58" s="80"/>
+      <c r="G58" s="80"/>
+      <c r="H58" s="80"/>
+      <c r="I58" s="28">
         <v>41061</v>
       </c>
-      <c r="J58" s="36"/>
-      <c r="K58" s="34"/>
-      <c r="L58" s="63"/>
-      <c r="M58" s="63"/>
-      <c r="N58" s="63"/>
-      <c r="O58" s="76"/>
-      <c r="P58" s="84"/>
+      <c r="J58" s="34"/>
+      <c r="K58" s="32"/>
+      <c r="L58" s="71"/>
+      <c r="M58" s="71"/>
+      <c r="N58" s="71"/>
+      <c r="O58" s="58"/>
+      <c r="P58" s="45"/>
     </row>
     <row r="59" spans="1:16">
-      <c r="A59" s="50">
+      <c r="A59" s="80">
         <v>2</v>
       </c>
-      <c r="B59" s="50" t="s">
+      <c r="B59" s="80" t="s">
         <v>89</v>
       </c>
-      <c r="C59" s="50" t="s">
+      <c r="C59" s="80" t="s">
         <v>72</v>
       </c>
-      <c r="D59" s="50" t="s">
+      <c r="D59" s="80" t="s">
         <v>90</v>
       </c>
-      <c r="E59" s="50" t="s">
+      <c r="E59" s="80" t="s">
         <v>91</v>
       </c>
-      <c r="F59" s="50" t="s">
+      <c r="F59" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="G59" s="50" t="s">
+      <c r="G59" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="H59" s="50" t="s">
+      <c r="H59" s="80" t="s">
         <v>40</v>
       </c>
-      <c r="I59" s="37">
+      <c r="I59" s="35">
         <v>41275</v>
       </c>
-      <c r="J59" s="37">
+      <c r="J59" s="35">
         <v>41334</v>
       </c>
-      <c r="K59" s="38">
+      <c r="K59" s="36">
         <v>41426</v>
       </c>
-      <c r="L59" s="63">
+      <c r="L59" s="71">
         <v>105000</v>
       </c>
-      <c r="M59" s="63">
+      <c r="M59" s="71">
         <v>165000</v>
       </c>
-      <c r="N59" s="63">
+      <c r="N59" s="71">
         <v>0</v>
       </c>
-      <c r="O59" s="76">
+      <c r="O59" s="58">
         <v>0.75</v>
       </c>
-      <c r="P59" s="84">
+      <c r="P59" s="45">
         <v>270000</v>
       </c>
     </row>
     <row r="60" spans="1:16">
-      <c r="A60" s="50"/>
-      <c r="B60" s="50"/>
-      <c r="C60" s="50"/>
-      <c r="D60" s="50"/>
-      <c r="E60" s="50"/>
-      <c r="F60" s="50"/>
-      <c r="G60" s="50"/>
-      <c r="H60" s="50"/>
-      <c r="I60" s="39">
+      <c r="A60" s="80"/>
+      <c r="B60" s="80"/>
+      <c r="C60" s="80"/>
+      <c r="D60" s="80"/>
+      <c r="E60" s="80"/>
+      <c r="F60" s="80"/>
+      <c r="G60" s="80"/>
+      <c r="H60" s="80"/>
+      <c r="I60" s="37">
         <v>41275</v>
       </c>
-      <c r="J60" s="39">
+      <c r="J60" s="37">
         <v>41306</v>
       </c>
-      <c r="K60" s="40">
+      <c r="K60" s="38">
         <v>41365</v>
       </c>
-      <c r="L60" s="63"/>
-      <c r="M60" s="63"/>
-      <c r="N60" s="63"/>
-      <c r="O60" s="76"/>
-      <c r="P60" s="84"/>
+      <c r="L60" s="71"/>
+      <c r="M60" s="71"/>
+      <c r="N60" s="71"/>
+      <c r="O60" s="58"/>
+      <c r="P60" s="45"/>
     </row>
     <row r="61" spans="1:16">
-      <c r="A61" s="51">
+      <c r="A61" s="81">
         <v>3</v>
       </c>
-      <c r="B61" s="51" t="s">
+      <c r="B61" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="C61" s="51" t="s">
+      <c r="C61" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D61" s="51" t="s">
+      <c r="D61" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="E61" s="51" t="s">
+      <c r="E61" s="81" t="s">
         <v>93</v>
       </c>
-      <c r="F61" s="51" t="s">
+      <c r="F61" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="G61" s="51" t="s">
+      <c r="G61" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="H61" s="51" t="s">
+      <c r="H61" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="I61" s="41">
+      <c r="I61" s="39">
         <v>41061</v>
       </c>
-      <c r="J61" s="41">
+      <c r="J61" s="39">
         <v>41426</v>
       </c>
-      <c r="K61" s="41">
+      <c r="K61" s="39">
         <v>41518</v>
       </c>
-      <c r="L61" s="64">
+      <c r="L61" s="61">
         <v>117600</v>
       </c>
-      <c r="M61" s="66">
+      <c r="M61" s="63">
         <v>184800</v>
       </c>
-      <c r="N61" s="64">
+      <c r="N61" s="61">
         <v>0</v>
       </c>
-      <c r="O61" s="77">
+      <c r="O61" s="49">
         <v>0.33</v>
       </c>
-      <c r="P61" s="85">
+      <c r="P61" s="46">
         <v>302400</v>
       </c>
     </row>
     <row r="62" spans="1:16">
-      <c r="A62" s="52"/>
-      <c r="B62" s="52"/>
-      <c r="C62" s="52"/>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="52"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="39">
+      <c r="A62" s="82"/>
+      <c r="B62" s="82"/>
+      <c r="C62" s="82"/>
+      <c r="D62" s="82"/>
+      <c r="E62" s="82"/>
+      <c r="F62" s="82"/>
+      <c r="G62" s="82"/>
+      <c r="H62" s="82"/>
+      <c r="I62" s="37">
         <v>41061</v>
       </c>
-      <c r="J62" s="39">
+      <c r="J62" s="37">
         <v>41365</v>
       </c>
-      <c r="K62" s="42"/>
-      <c r="L62" s="65"/>
-      <c r="M62" s="67"/>
-      <c r="N62" s="65"/>
-      <c r="O62" s="78"/>
-      <c r="P62" s="86"/>
+      <c r="K62" s="40"/>
+      <c r="L62" s="62"/>
+      <c r="M62" s="64"/>
+      <c r="N62" s="62"/>
+      <c r="O62" s="50"/>
+      <c r="P62" s="47"/>
     </row>
     <row r="63" spans="1:16">
-      <c r="A63" s="51">
+      <c r="A63" s="81">
         <v>2</v>
       </c>
-      <c r="B63" s="51" t="s">
+      <c r="B63" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="C63" s="51" t="s">
+      <c r="C63" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D63" s="51" t="s">
+      <c r="D63" s="81" t="s">
         <v>94</v>
       </c>
-      <c r="E63" s="51" t="s">
+      <c r="E63" s="81" t="s">
         <v>95</v>
       </c>
-      <c r="F63" s="51" t="s">
+      <c r="F63" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="G63" s="51" t="s">
+      <c r="G63" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="H63" s="51" t="s">
+      <c r="H63" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="I63" s="41">
+      <c r="I63" s="39">
         <v>40909</v>
       </c>
-      <c r="J63" s="41">
+      <c r="J63" s="39">
         <v>40909</v>
       </c>
-      <c r="K63" s="43">
+      <c r="K63" s="41">
         <v>40909</v>
       </c>
-      <c r="L63" s="64">
+      <c r="L63" s="61">
         <v>67200</v>
       </c>
-      <c r="M63" s="64">
+      <c r="M63" s="61">
         <v>124800</v>
       </c>
-      <c r="N63" s="64">
+      <c r="N63" s="61">
         <v>0</v>
       </c>
-      <c r="O63" s="77">
+      <c r="O63" s="49">
         <v>1</v>
       </c>
-      <c r="P63" s="85">
+      <c r="P63" s="46">
         <v>192000</v>
       </c>
     </row>
     <row r="64" spans="1:16">
-      <c r="A64" s="52"/>
-      <c r="B64" s="52"/>
-      <c r="C64" s="52"/>
-      <c r="D64" s="52"/>
-      <c r="E64" s="52"/>
-      <c r="F64" s="52"/>
-      <c r="G64" s="52"/>
-      <c r="H64" s="52"/>
-      <c r="I64" s="39">
+      <c r="A64" s="82"/>
+      <c r="B64" s="82"/>
+      <c r="C64" s="82"/>
+      <c r="D64" s="82"/>
+      <c r="E64" s="82"/>
+      <c r="F64" s="82"/>
+      <c r="G64" s="82"/>
+      <c r="H64" s="82"/>
+      <c r="I64" s="37">
         <v>40878</v>
       </c>
-      <c r="J64" s="39">
+      <c r="J64" s="37">
         <v>40878</v>
       </c>
-      <c r="K64" s="40">
+      <c r="K64" s="38">
         <v>40909</v>
       </c>
-      <c r="L64" s="65"/>
-      <c r="M64" s="65"/>
-      <c r="N64" s="65"/>
-      <c r="O64" s="78"/>
-      <c r="P64" s="86"/>
+      <c r="L64" s="62"/>
+      <c r="M64" s="62"/>
+      <c r="N64" s="62"/>
+      <c r="O64" s="50"/>
+      <c r="P64" s="47"/>
     </row>
     <row r="65" spans="1:16">
-      <c r="A65" s="51">
+      <c r="A65" s="81">
         <v>2</v>
       </c>
-      <c r="B65" s="51" t="s">
+      <c r="B65" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="C65" s="51" t="s">
+      <c r="C65" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D65" s="51" t="s">
+      <c r="D65" s="81" t="s">
         <v>96</v>
       </c>
-      <c r="E65" s="51" t="s">
+      <c r="E65" s="81" t="s">
         <v>97</v>
       </c>
-      <c r="F65" s="51" t="s">
+      <c r="F65" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="G65" s="51" t="s">
+      <c r="G65" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="H65" s="51" t="s">
+      <c r="H65" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="I65" s="41">
+      <c r="I65" s="39">
         <v>40909</v>
       </c>
-      <c r="J65" s="41">
+      <c r="J65" s="39">
         <v>40909</v>
       </c>
-      <c r="K65" s="43">
+      <c r="K65" s="41">
         <v>40909</v>
       </c>
-      <c r="L65" s="64">
+      <c r="L65" s="61">
         <v>22400</v>
       </c>
-      <c r="M65" s="64">
+      <c r="M65" s="61">
         <v>31200</v>
       </c>
-      <c r="N65" s="64">
+      <c r="N65" s="61">
         <v>0</v>
       </c>
-      <c r="O65" s="77">
+      <c r="O65" s="49">
         <v>1</v>
       </c>
-      <c r="P65" s="85">
+      <c r="P65" s="46">
         <v>53600</v>
       </c>
     </row>
     <row r="66" spans="1:16">
-      <c r="A66" s="52"/>
-      <c r="B66" s="52"/>
-      <c r="C66" s="52"/>
-      <c r="D66" s="52"/>
-      <c r="E66" s="52"/>
-      <c r="F66" s="52"/>
-      <c r="G66" s="52"/>
-      <c r="H66" s="52"/>
-      <c r="I66" s="39">
+      <c r="A66" s="82"/>
+      <c r="B66" s="82"/>
+      <c r="C66" s="82"/>
+      <c r="D66" s="82"/>
+      <c r="E66" s="82"/>
+      <c r="F66" s="82"/>
+      <c r="G66" s="82"/>
+      <c r="H66" s="82"/>
+      <c r="I66" s="37">
         <v>40878</v>
       </c>
-      <c r="J66" s="39">
+      <c r="J66" s="37">
         <v>40878</v>
       </c>
-      <c r="K66" s="40">
+      <c r="K66" s="38">
         <v>40909</v>
       </c>
-      <c r="L66" s="65"/>
-      <c r="M66" s="65"/>
-      <c r="N66" s="65"/>
-      <c r="O66" s="78"/>
-      <c r="P66" s="86"/>
+      <c r="L66" s="62"/>
+      <c r="M66" s="62"/>
+      <c r="N66" s="62"/>
+      <c r="O66" s="50"/>
+      <c r="P66" s="47"/>
     </row>
     <row r="67" spans="1:16">
-      <c r="A67" s="51">
+      <c r="A67" s="81">
         <v>2</v>
       </c>
-      <c r="B67" s="51" t="s">
+      <c r="B67" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="C67" s="51" t="s">
+      <c r="C67" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D67" s="51" t="s">
+      <c r="D67" s="81" t="s">
         <v>98</v>
       </c>
-      <c r="E67" s="51" t="s">
+      <c r="E67" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="F67" s="51" t="s">
+      <c r="F67" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="G67" s="51" t="s">
+      <c r="G67" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="H67" s="51">
+      <c r="H67" s="81">
         <v>737</v>
       </c>
-      <c r="I67" s="41">
+      <c r="I67" s="39">
         <v>41061</v>
       </c>
-      <c r="J67" s="41">
+      <c r="J67" s="39">
         <v>41122</v>
       </c>
-      <c r="K67" s="43">
+      <c r="K67" s="41">
         <v>41275</v>
       </c>
-      <c r="L67" s="64">
+      <c r="L67" s="61">
         <v>114400</v>
       </c>
-      <c r="M67" s="64">
+      <c r="M67" s="61">
         <v>0</v>
       </c>
-      <c r="N67" s="64">
+      <c r="N67" s="61">
         <v>17680</v>
       </c>
-      <c r="O67" s="77">
+      <c r="O67" s="49">
         <v>1</v>
       </c>
-      <c r="P67" s="85">
+      <c r="P67" s="46">
         <v>132080</v>
       </c>
     </row>
     <row r="68" spans="1:16">
-      <c r="A68" s="52"/>
-      <c r="B68" s="52"/>
-      <c r="C68" s="52"/>
-      <c r="D68" s="52"/>
-      <c r="E68" s="52"/>
-      <c r="F68" s="52"/>
-      <c r="G68" s="52"/>
-      <c r="H68" s="52"/>
-      <c r="I68" s="39">
+      <c r="A68" s="82"/>
+      <c r="B68" s="82"/>
+      <c r="C68" s="82"/>
+      <c r="D68" s="82"/>
+      <c r="E68" s="82"/>
+      <c r="F68" s="82"/>
+      <c r="G68" s="82"/>
+      <c r="H68" s="82"/>
+      <c r="I68" s="37">
         <v>41061</v>
       </c>
-      <c r="J68" s="39">
+      <c r="J68" s="37">
         <v>41061</v>
       </c>
-      <c r="K68" s="40">
+      <c r="K68" s="38">
         <v>41091</v>
       </c>
-      <c r="L68" s="65"/>
-      <c r="M68" s="65"/>
-      <c r="N68" s="65"/>
-      <c r="O68" s="78"/>
-      <c r="P68" s="86"/>
+      <c r="L68" s="62"/>
+      <c r="M68" s="62"/>
+      <c r="N68" s="62"/>
+      <c r="O68" s="50"/>
+      <c r="P68" s="47"/>
     </row>
     <row r="69" spans="1:16">
-      <c r="A69" s="51">
+      <c r="A69" s="81">
         <v>2</v>
       </c>
-      <c r="B69" s="51" t="s">
+      <c r="B69" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="C69" s="51" t="s">
+      <c r="C69" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="D69" s="51" t="s">
+      <c r="D69" s="81" t="s">
         <v>100</v>
       </c>
-      <c r="E69" s="51" t="s">
+      <c r="E69" s="81" t="s">
         <v>93</v>
       </c>
-      <c r="F69" s="51" t="s">
+      <c r="F69" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="G69" s="51" t="s">
+      <c r="G69" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="H69" s="51" t="s">
+      <c r="H69" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="I69" s="37">
+      <c r="I69" s="35">
         <v>41061</v>
       </c>
-      <c r="J69" s="37">
+      <c r="J69" s="35">
         <v>41153</v>
       </c>
-      <c r="K69" s="38">
+      <c r="K69" s="36">
         <v>41306</v>
       </c>
-      <c r="L69" s="66">
+      <c r="L69" s="63">
         <v>77700</v>
       </c>
-      <c r="M69" s="66">
+      <c r="M69" s="63">
         <v>144300</v>
       </c>
-      <c r="N69" s="66">
+      <c r="N69" s="63">
         <v>0</v>
       </c>
-      <c r="O69" s="79">
+      <c r="O69" s="51">
         <v>1</v>
       </c>
-      <c r="P69" s="85">
+      <c r="P69" s="46">
         <v>222000</v>
       </c>
     </row>
     <row r="70" spans="1:16">
-      <c r="A70" s="52"/>
-      <c r="B70" s="52"/>
-      <c r="C70" s="52"/>
-      <c r="D70" s="52"/>
-      <c r="E70" s="52"/>
-      <c r="F70" s="52"/>
-      <c r="G70" s="52"/>
-      <c r="H70" s="52"/>
-      <c r="I70" s="39">
+      <c r="A70" s="82"/>
+      <c r="B70" s="82"/>
+      <c r="C70" s="82"/>
+      <c r="D70" s="82"/>
+      <c r="E70" s="82"/>
+      <c r="F70" s="82"/>
+      <c r="G70" s="82"/>
+      <c r="H70" s="82"/>
+      <c r="I70" s="37">
         <v>41061</v>
       </c>
-      <c r="J70" s="44">
+      <c r="J70" s="92">
         <v>41183</v>
       </c>
-      <c r="K70" s="40">
+      <c r="K70" s="38">
         <v>41244</v>
       </c>
-      <c r="L70" s="67"/>
-      <c r="M70" s="67"/>
-      <c r="N70" s="67"/>
-      <c r="O70" s="80"/>
-      <c r="P70" s="86"/>
+      <c r="L70" s="64"/>
+      <c r="M70" s="64"/>
+      <c r="N70" s="64"/>
+      <c r="O70" s="52"/>
+      <c r="P70" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="446">
-    <mergeCell ref="P59:P60"/>
-    <mergeCell ref="P61:P62"/>
-    <mergeCell ref="P63:P64"/>
-    <mergeCell ref="P65:P66"/>
-    <mergeCell ref="P67:P68"/>
-    <mergeCell ref="P69:P70"/>
-    <mergeCell ref="P41:P42"/>
-    <mergeCell ref="P43:P44"/>
-    <mergeCell ref="P45:P46"/>
-    <mergeCell ref="P47:P48"/>
-    <mergeCell ref="P49:P50"/>
-    <mergeCell ref="P51:P52"/>
-    <mergeCell ref="P53:P54"/>
-    <mergeCell ref="P55:P56"/>
-    <mergeCell ref="P57:P58"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:P1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="D51:D52"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="D57:D58"/>
+    <mergeCell ref="D59:D60"/>
+    <mergeCell ref="D61:D62"/>
+    <mergeCell ref="D63:D64"/>
+    <mergeCell ref="D65:D66"/>
+    <mergeCell ref="D67:D68"/>
+    <mergeCell ref="D69:D70"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="G43:G44"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="G51:G52"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="G55:G56"/>
+    <mergeCell ref="G57:G58"/>
+    <mergeCell ref="G59:G60"/>
+    <mergeCell ref="G61:G62"/>
+    <mergeCell ref="G63:G64"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="G67:G68"/>
+    <mergeCell ref="G69:G70"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="H37:H38"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="H41:H42"/>
+    <mergeCell ref="H43:H44"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="H49:H50"/>
+    <mergeCell ref="H51:H52"/>
+    <mergeCell ref="H53:H54"/>
+    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="H57:H58"/>
+    <mergeCell ref="H59:H60"/>
+    <mergeCell ref="H61:H62"/>
+    <mergeCell ref="H63:H64"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="H67:H68"/>
+    <mergeCell ref="H69:H70"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="L33:L34"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="L37:L38"/>
+    <mergeCell ref="L39:L40"/>
+    <mergeCell ref="L41:L42"/>
+    <mergeCell ref="L43:L44"/>
+    <mergeCell ref="L45:L46"/>
+    <mergeCell ref="L47:L48"/>
+    <mergeCell ref="L49:L50"/>
+    <mergeCell ref="L51:L52"/>
+    <mergeCell ref="L53:L54"/>
+    <mergeCell ref="L55:L56"/>
+    <mergeCell ref="L57:L58"/>
+    <mergeCell ref="L59:L60"/>
+    <mergeCell ref="L61:L62"/>
+    <mergeCell ref="L63:L64"/>
+    <mergeCell ref="L65:L66"/>
+    <mergeCell ref="L67:L68"/>
+    <mergeCell ref="L69:L70"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="M13:M14"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="M25:M26"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="M33:M34"/>
+    <mergeCell ref="M35:M36"/>
+    <mergeCell ref="M37:M38"/>
+    <mergeCell ref="M39:M40"/>
+    <mergeCell ref="M41:M42"/>
+    <mergeCell ref="M43:M44"/>
+    <mergeCell ref="M45:M46"/>
+    <mergeCell ref="M47:M48"/>
+    <mergeCell ref="M49:M50"/>
+    <mergeCell ref="M51:M52"/>
+    <mergeCell ref="M53:M54"/>
+    <mergeCell ref="M55:M56"/>
+    <mergeCell ref="M57:M58"/>
+    <mergeCell ref="M59:M60"/>
+    <mergeCell ref="M61:M62"/>
+    <mergeCell ref="M63:M64"/>
+    <mergeCell ref="M65:M66"/>
+    <mergeCell ref="M67:M68"/>
+    <mergeCell ref="M69:M70"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="N25:N26"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="N33:N34"/>
+    <mergeCell ref="N35:N36"/>
+    <mergeCell ref="N37:N38"/>
+    <mergeCell ref="N39:N40"/>
+    <mergeCell ref="N41:N42"/>
+    <mergeCell ref="N43:N44"/>
+    <mergeCell ref="N45:N46"/>
+    <mergeCell ref="N47:N48"/>
+    <mergeCell ref="N49:N50"/>
+    <mergeCell ref="N51:N52"/>
+    <mergeCell ref="N53:N54"/>
+    <mergeCell ref="N55:N56"/>
+    <mergeCell ref="N57:N58"/>
+    <mergeCell ref="N59:N60"/>
+    <mergeCell ref="N61:N62"/>
+    <mergeCell ref="N63:N64"/>
+    <mergeCell ref="N65:N66"/>
+    <mergeCell ref="N67:N68"/>
+    <mergeCell ref="N69:N70"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="O15:O16"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="O21:O22"/>
+    <mergeCell ref="O23:O24"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="O29:O30"/>
+    <mergeCell ref="O31:O32"/>
+    <mergeCell ref="O33:O34"/>
+    <mergeCell ref="O35:O36"/>
+    <mergeCell ref="O37:O38"/>
+    <mergeCell ref="O39:O40"/>
+    <mergeCell ref="O41:O42"/>
+    <mergeCell ref="O43:O44"/>
+    <mergeCell ref="O45:O46"/>
+    <mergeCell ref="O47:O48"/>
+    <mergeCell ref="O49:O50"/>
+    <mergeCell ref="O51:O52"/>
+    <mergeCell ref="O53:O54"/>
+    <mergeCell ref="O55:O56"/>
+    <mergeCell ref="O57:O58"/>
+    <mergeCell ref="O59:O60"/>
     <mergeCell ref="O61:O62"/>
     <mergeCell ref="O63:O64"/>
     <mergeCell ref="O65:O66"/>
@@ -3983,413 +4387,21 @@
     <mergeCell ref="P35:P36"/>
     <mergeCell ref="P37:P38"/>
     <mergeCell ref="P39:P40"/>
-    <mergeCell ref="O43:O44"/>
-    <mergeCell ref="O45:O46"/>
-    <mergeCell ref="O47:O48"/>
-    <mergeCell ref="O49:O50"/>
-    <mergeCell ref="O51:O52"/>
-    <mergeCell ref="O53:O54"/>
-    <mergeCell ref="O55:O56"/>
-    <mergeCell ref="O57:O58"/>
-    <mergeCell ref="O59:O60"/>
-    <mergeCell ref="N63:N64"/>
-    <mergeCell ref="N65:N66"/>
-    <mergeCell ref="N67:N68"/>
-    <mergeCell ref="N69:N70"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="O21:O22"/>
-    <mergeCell ref="O23:O24"/>
-    <mergeCell ref="O25:O26"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="O29:O30"/>
-    <mergeCell ref="O31:O32"/>
-    <mergeCell ref="O33:O34"/>
-    <mergeCell ref="O35:O36"/>
-    <mergeCell ref="O37:O38"/>
-    <mergeCell ref="O39:O40"/>
-    <mergeCell ref="O41:O42"/>
-    <mergeCell ref="N45:N46"/>
-    <mergeCell ref="N47:N48"/>
-    <mergeCell ref="N49:N50"/>
-    <mergeCell ref="N51:N52"/>
-    <mergeCell ref="N53:N54"/>
-    <mergeCell ref="N55:N56"/>
-    <mergeCell ref="N57:N58"/>
-    <mergeCell ref="N59:N60"/>
-    <mergeCell ref="N61:N62"/>
-    <mergeCell ref="M65:M66"/>
-    <mergeCell ref="M67:M68"/>
-    <mergeCell ref="M69:M70"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="N31:N32"/>
-    <mergeCell ref="N33:N34"/>
-    <mergeCell ref="N35:N36"/>
-    <mergeCell ref="N37:N38"/>
-    <mergeCell ref="N39:N40"/>
-    <mergeCell ref="N41:N42"/>
-    <mergeCell ref="N43:N44"/>
-    <mergeCell ref="M47:M48"/>
-    <mergeCell ref="M49:M50"/>
-    <mergeCell ref="M51:M52"/>
-    <mergeCell ref="M53:M54"/>
-    <mergeCell ref="M55:M56"/>
-    <mergeCell ref="M57:M58"/>
-    <mergeCell ref="M59:M60"/>
-    <mergeCell ref="M61:M62"/>
-    <mergeCell ref="M63:M64"/>
-    <mergeCell ref="L67:L68"/>
-    <mergeCell ref="L69:L70"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="M13:M14"/>
-    <mergeCell ref="M15:M16"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="M25:M26"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="M33:M34"/>
-    <mergeCell ref="M35:M36"/>
-    <mergeCell ref="M37:M38"/>
-    <mergeCell ref="M39:M40"/>
-    <mergeCell ref="M41:M42"/>
-    <mergeCell ref="M43:M44"/>
-    <mergeCell ref="M45:M46"/>
-    <mergeCell ref="L49:L50"/>
-    <mergeCell ref="L51:L52"/>
-    <mergeCell ref="L53:L54"/>
-    <mergeCell ref="L55:L56"/>
-    <mergeCell ref="L57:L58"/>
-    <mergeCell ref="L59:L60"/>
-    <mergeCell ref="L61:L62"/>
-    <mergeCell ref="L63:L64"/>
-    <mergeCell ref="L65:L66"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="L33:L34"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="L37:L38"/>
-    <mergeCell ref="L39:L40"/>
-    <mergeCell ref="L41:L42"/>
-    <mergeCell ref="L43:L44"/>
-    <mergeCell ref="L45:L46"/>
-    <mergeCell ref="L47:L48"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="H53:H54"/>
-    <mergeCell ref="H55:H56"/>
-    <mergeCell ref="H57:H58"/>
-    <mergeCell ref="H59:H60"/>
-    <mergeCell ref="H61:H62"/>
-    <mergeCell ref="H63:H64"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="H67:H68"/>
-    <mergeCell ref="H69:H70"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="H37:H38"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="H41:H42"/>
-    <mergeCell ref="H43:H44"/>
-    <mergeCell ref="H45:H46"/>
-    <mergeCell ref="H47:H48"/>
-    <mergeCell ref="H49:H50"/>
-    <mergeCell ref="H51:H52"/>
-    <mergeCell ref="G55:G56"/>
-    <mergeCell ref="G57:G58"/>
-    <mergeCell ref="G59:G60"/>
-    <mergeCell ref="G61:G62"/>
-    <mergeCell ref="G63:G64"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="G67:G68"/>
-    <mergeCell ref="G69:G70"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="G43:G44"/>
-    <mergeCell ref="G45:G46"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="G49:G50"/>
-    <mergeCell ref="G51:G52"/>
-    <mergeCell ref="G53:G54"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="D61:D62"/>
-    <mergeCell ref="D63:D64"/>
-    <mergeCell ref="D65:D66"/>
-    <mergeCell ref="D67:D68"/>
-    <mergeCell ref="D69:D70"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="D57:D58"/>
-    <mergeCell ref="D59:D60"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="A67:A68"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="A63:A64"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:P1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="P59:P60"/>
+    <mergeCell ref="P61:P62"/>
+    <mergeCell ref="P63:P64"/>
+    <mergeCell ref="P65:P66"/>
+    <mergeCell ref="P67:P68"/>
+    <mergeCell ref="P69:P70"/>
+    <mergeCell ref="P41:P42"/>
+    <mergeCell ref="P43:P44"/>
+    <mergeCell ref="P45:P46"/>
+    <mergeCell ref="P47:P48"/>
+    <mergeCell ref="P49:P50"/>
+    <mergeCell ref="P51:P52"/>
+    <mergeCell ref="P53:P54"/>
+    <mergeCell ref="P55:P56"/>
+    <mergeCell ref="P57:P58"/>
   </mergeCells>
   <conditionalFormatting sqref="K4">
     <cfRule type="expression" dxfId="9" priority="8">

</xml_diff>